<commit_message>
Bump CEB-GNRD firmware to 2.01 and refresh project guides
</commit_message>
<xml_diff>
--- a/meta-ctopai/port_guide.xlsx
+++ b/meta-ctopai/port_guide.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="端口映射" sheetId="1" r:id="R9722541e1f2e44b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="端口映射" sheetId="1" r:id="Rf2354700f7004d6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,7 +89,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +104,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EEF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -132,7 +137,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -183,6 +188,17 @@
     <x:xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -192,8 +208,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HardwarePorts" displayName="HardwarePorts" ref="A4:H163" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:H163"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HardwarePorts" displayName="HardwarePorts" ref="A4:H164" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:H164"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="类别"/>
     <x:tableColumn id="2" name="接口 / 信号"/>
@@ -603,7 +619,7 @@
         <x:v>输入；低有效</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>检测机箱电源按键</x:v>
+        <x:v>仅通知 BMC 实体按键状态；不转发电源动作</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
         <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
@@ -741,7 +757,7 @@
       <x:c r="I14"/>
       <x:c r="J14"/>
     </x:row>
-    <x:row r="15" ht="66" customHeight="1">
+    <x:row r="15" ht="94" customHeight="1">
       <x:c r="A15" s="11" t="str">
         <x:v>GPIO / 状态线</x:v>
       </x:c>
@@ -759,10 +775,10 @@
         <x:v>输入；低有效</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str">
-        <x:v>检测 UID 按键</x:v>
+        <x:v>UID 定位；连续长按 5 秒请求 BMC 重启</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml；recipes-phosphor/buttons/files/0001-ceb-gnrd-uid-long-press-bmc-reboot.patch</x:v>
       </x:c>
       <x:c r="I15"/>
       <x:c r="J15"/>
@@ -1360,7 +1376,7 @@
         <x:v>ADC1 channel 7 / Index 15</x:v>
       </x:c>
       <x:c r="F37" s="11" t="str">
-        <x:v>内部参考 2.5 V；ScaleFactor=1.0；电压换算：ADC 输入电压 / ScaleFactor</x:v>
+        <x:v>内部参考 2.5 V；ScaleFactor=0.5；电压换算：ADC 输入电压 / ScaleFactor</x:v>
       </x:c>
       <x:c r="G37" s="11" t="str">
         <x:v>采集 D3V0_BAT0</x:v>
@@ -2116,7 +2132,7 @@
         <x:v>物理 I2C8 = DT i2c7；0x58 / 0x59 / 0x5a</x:v>
       </x:c>
       <x:c r="F64" s="11" t="str">
-        <x:v>Linux 启用；pinctrl_i2c8_default</x:v>
+        <x:v>Linux 启用；pinctrl_i2c8_default；clock-frequency=100000（100 kbit/s）</x:v>
       </x:c>
       <x:c r="G64" s="11" t="str">
         <x:v>板级 I2C 通信</x:v>
@@ -2144,7 +2160,7 @@
         <x:v>物理 I2C8 = DT i2c7；0x58 / 0x59 / 0x5a</x:v>
       </x:c>
       <x:c r="F65" s="11" t="str">
-        <x:v>Linux 启用；pinctrl_i2c8_default</x:v>
+        <x:v>Linux 启用；pinctrl_i2c8_default；clock-frequency=100000（100 kbit/s）</x:v>
       </x:c>
       <x:c r="G65" s="11" t="str">
         <x:v>板级 I2C 通信</x:v>
@@ -2603,7 +2619,7 @@
       <x:c r="I81"/>
       <x:c r="J81"/>
     </x:row>
-    <x:row r="82" ht="66" customHeight="1">
+    <x:row r="82" ht="80" customHeight="1">
       <x:c r="A82" s="19" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2626,12 +2642,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H82" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I82"/>
       <x:c r="J82"/>
     </x:row>
-    <x:row r="83" ht="66" customHeight="1">
+    <x:row r="83" ht="80" customHeight="1">
       <x:c r="A83" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2654,12 +2670,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H83" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I83"/>
       <x:c r="J83"/>
     </x:row>
-    <x:row r="84" ht="66" customHeight="1">
+    <x:row r="84" ht="80" customHeight="1">
       <x:c r="A84" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2682,12 +2698,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H84" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I84"/>
       <x:c r="J84"/>
     </x:row>
-    <x:row r="85" ht="66" customHeight="1">
+    <x:row r="85" ht="80" customHeight="1">
       <x:c r="A85" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2710,12 +2726,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H85" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I85"/>
       <x:c r="J85"/>
     </x:row>
-    <x:row r="86" ht="66" customHeight="1">
+    <x:row r="86" ht="80" customHeight="1">
       <x:c r="A86" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2738,12 +2754,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H86" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I86"/>
       <x:c r="J86"/>
     </x:row>
-    <x:row r="87" ht="66" customHeight="1">
+    <x:row r="87" ht="80" customHeight="1">
       <x:c r="A87" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2766,12 +2782,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H87" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I87"/>
       <x:c r="J87"/>
     </x:row>
-    <x:row r="88" ht="66" customHeight="1">
+    <x:row r="88" ht="80" customHeight="1">
       <x:c r="A88" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2794,12 +2810,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H88" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I88"/>
       <x:c r="J88"/>
     </x:row>
-    <x:row r="89" ht="66" customHeight="1">
+    <x:row r="89" ht="80" customHeight="1">
       <x:c r="A89" s="11" t="str">
         <x:v>eSPI</x:v>
       </x:c>
@@ -2822,12 +2838,12 @@
         <x:v>主机与 BMC 的 eSPI 连接</x:v>
       </x:c>
       <x:c r="H89" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-ceb-gnrd-enable-espi-peripheral.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；0001-soc-aspeed-add-AST2600-eSPI-peripheral-ready-driver.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I89"/>
       <x:c r="J89"/>
     </x:row>
-    <x:row r="90" ht="66" customHeight="1">
+    <x:row r="90" ht="80" customHeight="1">
       <x:c r="A90" s="19" t="str">
         <x:v>UART</x:v>
       </x:c>
@@ -2844,18 +2860,18 @@
         <x:v>BMC_CPU_SOL_TXD</x:v>
       </x:c>
       <x:c r="F90" s="18" t="str">
-        <x:v>未复用为 TXD3；保留 GPIO 输入</x:v>
+        <x:v>UART3 TX/RX 启用；pinctrl_txd3_default / pinctrl_rxd3_default；115200 baud；ttyS2</x:v>
       </x:c>
       <x:c r="G90" s="18" t="str">
-        <x:v>UART3 TX 引脚保留；不用于 SOL</x:v>
+        <x:v>默认物理主机 SOL 发送</x:v>
       </x:c>
       <x:c r="H90" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；conf/machine/ceb-gnrd.conf；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；conf/machine/ceb-gnrd.conf；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）；recipes-phosphor/console/files/server.ttyS2.conf</x:v>
       </x:c>
       <x:c r="I90"/>
       <x:c r="J90"/>
     </x:row>
-    <x:row r="91" ht="66" customHeight="1">
+    <x:row r="91" ht="80" customHeight="1">
       <x:c r="A91" s="11" t="str">
         <x:v>UART</x:v>
       </x:c>
@@ -2872,13 +2888,13 @@
         <x:v>BMC_CPU_SOL_RXD</x:v>
       </x:c>
       <x:c r="F91" s="11" t="str">
-        <x:v>UART3 启用；仅 pinctrl_rxd3_default</x:v>
+        <x:v>UART3 TX/RX 启用；pinctrl_txd3_default / pinctrl_rxd3_default；115200 baud；ttyS2</x:v>
       </x:c>
       <x:c r="G91" s="11" t="str">
-        <x:v>UART3 接收输入；不用于 SOL</x:v>
+        <x:v>默认物理主机 SOL 接收</x:v>
       </x:c>
       <x:c r="H91" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；conf/machine/ceb-gnrd.conf；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；conf/machine/ceb-gnrd.conf；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）；recipes-phosphor/console/files/server.ttyS2.conf</x:v>
       </x:c>
       <x:c r="I91"/>
       <x:c r="J91"/>
@@ -3051,7 +3067,7 @@
       <x:c r="I97"/>
       <x:c r="J97"/>
     </x:row>
-    <x:row r="98" ht="80" customHeight="1">
+    <x:row r="98" ht="94" customHeight="1">
       <x:c r="A98" s="19" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3065,21 +3081,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E98" s="18" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F98" s="18" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G98" s="18" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H98" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I98"/>
       <x:c r="J98"/>
     </x:row>
-    <x:row r="99" ht="80" customHeight="1">
+    <x:row r="99" ht="94" customHeight="1">
       <x:c r="A99" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3093,21 +3109,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E99" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F99" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G99" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H99" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I99"/>
       <x:c r="J99"/>
     </x:row>
-    <x:row r="100" ht="80" customHeight="1">
+    <x:row r="100" ht="94" customHeight="1">
       <x:c r="A100" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3121,21 +3137,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E100" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F100" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G100" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H100" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I100"/>
       <x:c r="J100"/>
     </x:row>
-    <x:row r="101" ht="80" customHeight="1">
+    <x:row r="101" ht="94" customHeight="1">
       <x:c r="A101" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3149,21 +3165,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E101" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F101" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G101" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H101" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I101"/>
       <x:c r="J101"/>
     </x:row>
-    <x:row r="102" ht="80" customHeight="1">
+    <x:row r="102" ht="94" customHeight="1">
       <x:c r="A102" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3177,21 +3193,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E102" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F102" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G102" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H102" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I102"/>
       <x:c r="J102"/>
     </x:row>
-    <x:row r="103" ht="80" customHeight="1">
+    <x:row r="103" ht="94" customHeight="1">
       <x:c r="A103" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3205,21 +3221,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E103" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F103" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G103" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H103" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I103"/>
       <x:c r="J103"/>
     </x:row>
-    <x:row r="104" ht="80" customHeight="1">
+    <x:row r="104" ht="94" customHeight="1">
       <x:c r="A104" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3233,21 +3249,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E104" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F104" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G104" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H104" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I104"/>
       <x:c r="J104"/>
     </x:row>
-    <x:row r="105" ht="80" customHeight="1">
+    <x:row r="105" ht="94" customHeight="1">
       <x:c r="A105" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3261,21 +3277,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E105" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F105" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G105" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H105" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I105"/>
       <x:c r="J105"/>
     </x:row>
-    <x:row r="106" ht="80" customHeight="1">
+    <x:row r="106" ht="94" customHeight="1">
       <x:c r="A106" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3289,21 +3305,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E106" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F106" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G106" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H106" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I106"/>
       <x:c r="J106"/>
     </x:row>
-    <x:row r="107" ht="80" customHeight="1">
+    <x:row r="107" ht="94" customHeight="1">
       <x:c r="A107" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3317,21 +3333,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E107" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F107" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G107" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H107" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I107"/>
       <x:c r="J107"/>
     </x:row>
-    <x:row r="108" ht="80" customHeight="1">
+    <x:row r="108" ht="94" customHeight="1">
       <x:c r="A108" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3345,21 +3361,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E108" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F108" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G108" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H108" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I108"/>
       <x:c r="J108"/>
     </x:row>
-    <x:row r="109" ht="80" customHeight="1">
+    <x:row r="109" ht="94" customHeight="1">
       <x:c r="A109" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3373,21 +3389,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E109" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F109" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G109" s="11" t="str">
         <x:v>BMC 独立管理网口</x:v>
       </x:c>
       <x:c r="H109" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I109"/>
       <x:c r="J109"/>
     </x:row>
-    <x:row r="110" ht="80" customHeight="1">
+    <x:row r="110" ht="94" customHeight="1">
       <x:c r="A110" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3401,21 +3417,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E110" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F110" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G110" s="11" t="str">
         <x:v>PHY 管理通信</x:v>
       </x:c>
       <x:c r="H110" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I110"/>
       <x:c r="J110"/>
     </x:row>
-    <x:row r="111" ht="80" customHeight="1">
+    <x:row r="111" ht="94" customHeight="1">
       <x:c r="A111" s="11" t="str">
         <x:v>Ethernet / PHY</x:v>
       </x:c>
@@ -3429,21 +3445,21 @@
         <x:v>RTL8211FS-CG</x:v>
       </x:c>
       <x:c r="E111" s="11" t="str">
-        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 2</x:v>
+        <x:v>mac1（物理 MAC2）/ Linux eth0；PHY 1</x:v>
       </x:c>
       <x:c r="F111" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；RGMII；pinctrl_rgmii2_default；MDIO1/PHY reg=2；PHY 复位由 CPLD 控制</x:v>
+        <x:v>Linux / U-Boot 启用；rgmii-id；pinctrl_rgmii2_default；MDIO1/PHY reg=1；PHY 复位由 CPLD 控制</x:v>
       </x:c>
       <x:c r="G111" s="11" t="str">
         <x:v>PHY 管理通信</x:v>
       </x:c>
       <x:c r="H111" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I111"/>
       <x:c r="J111"/>
     </x:row>
-    <x:row r="112" ht="80" customHeight="1">
+    <x:row r="112" ht="94" customHeight="1">
       <x:c r="A112" s="19" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3466,12 +3482,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H112" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I112"/>
       <x:c r="J112"/>
     </x:row>
-    <x:row r="113" ht="80" customHeight="1">
+    <x:row r="113" ht="94" customHeight="1">
       <x:c r="A113" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3494,12 +3510,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H113" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I113"/>
       <x:c r="J113"/>
     </x:row>
-    <x:row r="114" ht="80" customHeight="1">
+    <x:row r="114" ht="94" customHeight="1">
       <x:c r="A114" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3522,12 +3538,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H114" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I114"/>
       <x:c r="J114"/>
     </x:row>
-    <x:row r="115" ht="80" customHeight="1">
+    <x:row r="115" ht="94" customHeight="1">
       <x:c r="A115" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3550,12 +3566,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H115" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I115"/>
       <x:c r="J115"/>
     </x:row>
-    <x:row r="116" ht="80" customHeight="1">
+    <x:row r="116" ht="94" customHeight="1">
       <x:c r="A116" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3578,12 +3594,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H116" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I116"/>
       <x:c r="J116"/>
     </x:row>
-    <x:row r="117" ht="80" customHeight="1">
+    <x:row r="117" ht="94" customHeight="1">
       <x:c r="A117" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3606,12 +3622,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H117" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I117"/>
       <x:c r="J117"/>
     </x:row>
-    <x:row r="118" ht="80" customHeight="1">
+    <x:row r="118" ht="94" customHeight="1">
       <x:c r="A118" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3634,12 +3650,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H118" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I118"/>
       <x:c r="J118"/>
     </x:row>
-    <x:row r="119" ht="80" customHeight="1">
+    <x:row r="119" ht="94" customHeight="1">
       <x:c r="A119" s="11" t="str">
         <x:v>Ethernet / NC-SI</x:v>
       </x:c>
@@ -3662,12 +3678,12 @@
         <x:v>共享 NIC 的 NC-SI 管理链路</x:v>
       </x:c>
       <x:c r="H119" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；球位: Linux pinctrl-aspeed-g6.c（内核 SRCREV c0538446e769）</x:v>
       </x:c>
       <x:c r="I119"/>
       <x:c r="J119"/>
     </x:row>
-    <x:row r="120" ht="80" customHeight="1">
+    <x:row r="120" ht="94" customHeight="1">
       <x:c r="A120" s="19" t="str">
         <x:v>SPI1 / BIOS Flash</x:v>
       </x:c>
@@ -3690,12 +3706,12 @@
         <x:v>访问主机 BIOS Flash</x:v>
       </x:c>
       <x:c r="H120" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I120"/>
       <x:c r="J120"/>
     </x:row>
-    <x:row r="121" ht="80" customHeight="1">
+    <x:row r="121" ht="94" customHeight="1">
       <x:c r="A121" s="11" t="str">
         <x:v>SPI1 / BIOS Flash</x:v>
       </x:c>
@@ -3718,12 +3734,12 @@
         <x:v>访问主机 BIOS Flash</x:v>
       </x:c>
       <x:c r="H121" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I121"/>
       <x:c r="J121"/>
     </x:row>
-    <x:row r="122" ht="80" customHeight="1">
+    <x:row r="122" ht="94" customHeight="1">
       <x:c r="A122" s="11" t="str">
         <x:v>SPI1 / BIOS Flash</x:v>
       </x:c>
@@ -3746,12 +3762,12 @@
         <x:v>访问主机 BIOS Flash</x:v>
       </x:c>
       <x:c r="H122" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I122"/>
       <x:c r="J122"/>
     </x:row>
-    <x:row r="123" ht="80" customHeight="1">
+    <x:row r="123" ht="94" customHeight="1">
       <x:c r="A123" s="11" t="str">
         <x:v>SPI1 / BIOS Flash</x:v>
       </x:c>
@@ -3774,12 +3790,12 @@
         <x:v>访问主机 BIOS Flash</x:v>
       </x:c>
       <x:c r="H123" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I123"/>
       <x:c r="J123"/>
     </x:row>
-    <x:row r="124" ht="80" customHeight="1">
+    <x:row r="124" ht="94" customHeight="1">
       <x:c r="A124" s="11" t="str">
         <x:v>SPI1 / BIOS Flash</x:v>
       </x:c>
@@ -3802,12 +3818,12 @@
         <x:v>访问主机 BIOS Flash</x:v>
       </x:c>
       <x:c r="H124" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I124"/>
       <x:c r="J124"/>
     </x:row>
-    <x:row r="125" ht="80" customHeight="1">
+    <x:row r="125" ht="94" customHeight="1">
       <x:c r="A125" s="11" t="str">
         <x:v>SPI1 / BIOS Flash</x:v>
       </x:c>
@@ -3830,12 +3846,12 @@
         <x:v>访问主机 BIOS Flash</x:v>
       </x:c>
       <x:c r="H125" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I125"/>
       <x:c r="J125"/>
     </x:row>
-    <x:row r="126" ht="80" customHeight="1">
+    <x:row r="126" ht="94" customHeight="1">
       <x:c r="A126" s="19" t="str">
         <x:v>FMC / BMC Flash</x:v>
       </x:c>
@@ -3852,18 +3868,18 @@
         <x:v>FMC CS0</x:v>
       </x:c>
       <x:c r="F126" s="18" t="str">
-        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；FWSPID + FWQSPI；仅配置 CS0</x:v>
+        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；仅 FWQSPI；CS0/CLK/DQ0/DQ1 使用专用启动引脚；仅配置 CS0</x:v>
       </x:c>
       <x:c r="G126" s="18" t="str">
         <x:v>BMC 启动及固件存储</x:v>
       </x:c>
       <x:c r="H126" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I126"/>
       <x:c r="J126"/>
     </x:row>
-    <x:row r="127" ht="80" customHeight="1">
+    <x:row r="127" ht="94" customHeight="1">
       <x:c r="A127" s="11" t="str">
         <x:v>FMC / BMC Flash</x:v>
       </x:c>
@@ -3880,18 +3896,18 @@
         <x:v>FMC CS0</x:v>
       </x:c>
       <x:c r="F127" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；FWSPID + FWQSPI；仅配置 CS0</x:v>
+        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；仅 FWQSPI；CS0/CLK/DQ0/DQ1 使用专用启动引脚；仅配置 CS0</x:v>
       </x:c>
       <x:c r="G127" s="11" t="str">
         <x:v>BMC 启动及固件存储</x:v>
       </x:c>
       <x:c r="H127" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I127"/>
       <x:c r="J127"/>
     </x:row>
-    <x:row r="128" ht="80" customHeight="1">
+    <x:row r="128" ht="94" customHeight="1">
       <x:c r="A128" s="11" t="str">
         <x:v>FMC / BMC Flash</x:v>
       </x:c>
@@ -3908,18 +3924,18 @@
         <x:v>FMC CS0</x:v>
       </x:c>
       <x:c r="F128" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；FWSPID + FWQSPI；仅配置 CS0</x:v>
+        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；仅 FWQSPI；CS0/CLK/DQ0/DQ1 使用专用启动引脚；仅配置 CS0</x:v>
       </x:c>
       <x:c r="G128" s="11" t="str">
         <x:v>BMC 启动及固件存储</x:v>
       </x:c>
       <x:c r="H128" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I128"/>
       <x:c r="J128"/>
     </x:row>
-    <x:row r="129" ht="80" customHeight="1">
+    <x:row r="129" ht="94" customHeight="1">
       <x:c r="A129" s="11" t="str">
         <x:v>FMC / BMC Flash</x:v>
       </x:c>
@@ -3936,18 +3952,18 @@
         <x:v>FMC CS0</x:v>
       </x:c>
       <x:c r="F129" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；FWSPID + FWQSPI；仅配置 CS0</x:v>
+        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；仅 FWQSPI；CS0/CLK/DQ0/DQ1 使用专用启动引脚；仅配置 CS0</x:v>
       </x:c>
       <x:c r="G129" s="11" t="str">
         <x:v>BMC 启动及固件存储</x:v>
       </x:c>
       <x:c r="H129" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I129"/>
       <x:c r="J129"/>
     </x:row>
-    <x:row r="130" ht="80" customHeight="1">
+    <x:row r="130" ht="94" customHeight="1">
       <x:c r="A130" s="11" t="str">
         <x:v>FMC / BMC Flash</x:v>
       </x:c>
@@ -3964,18 +3980,18 @@
         <x:v>FMC CS0</x:v>
       </x:c>
       <x:c r="F130" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；FWSPID + FWQSPI；仅配置 CS0</x:v>
+        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；仅 FWQSPI；CS0/CLK/DQ0/DQ1 使用专用启动引脚；仅配置 CS0</x:v>
       </x:c>
       <x:c r="G130" s="11" t="str">
         <x:v>BMC 启动及固件存储</x:v>
       </x:c>
       <x:c r="H130" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I130"/>
       <x:c r="J130"/>
     </x:row>
-    <x:row r="131" ht="80" customHeight="1">
+    <x:row r="131" ht="94" customHeight="1">
       <x:c r="A131" s="11" t="str">
         <x:v>FMC / BMC Flash</x:v>
       </x:c>
@@ -3992,13 +4008,13 @@
         <x:v>FMC CS0</x:v>
       </x:c>
       <x:c r="F131" s="11" t="str">
-        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；FWSPID + FWQSPI；仅配置 CS0</x:v>
+        <x:v>Linux / U-Boot 启用；50 MHz 上限；RX/TX x4；仅 FWQSPI；CS0/CLK/DQ0/DQ1 使用专用启动引脚；仅配置 CS0</x:v>
       </x:c>
       <x:c r="G131" s="11" t="str">
         <x:v>BMC 启动及固件存储</x:v>
       </x:c>
       <x:c r="H131" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；引脚/器件: recipes-phosphor/configuration/files/ceb-gnrd-hardware-contract.yaml</x:v>
       </x:c>
       <x:c r="I131"/>
       <x:c r="J131"/>
@@ -4193,7 +4209,7 @@
       <x:c r="I138"/>
       <x:c r="J138"/>
     </x:row>
-    <x:row r="139" ht="42" customHeight="1">
+    <x:row r="139" ht="52" customHeight="1">
       <x:c r="A139" s="11" t="str">
         <x:v>I2C 器件</x:v>
       </x:c>
@@ -4210,18 +4226,18 @@
         <x:v>0x58</x:v>
       </x:c>
       <x:c r="F139" s="11" t="str">
-        <x:v>PMBus；vin / vout1 / pin / pout1 / temp2</x:v>
+        <x:v>PMBus 100 kbit/s；MEG 型号专用驱动，其余 generic pmbus；仅在位地址实例化</x:v>
       </x:c>
       <x:c r="G139" s="11" t="str">
-        <x:v>PSU 电压、电功率与温度采样</x:v>
+        <x:v>PSU 电压、电功率与温度采样；实际通道由模块决定</x:v>
       </x:c>
       <x:c r="H139" s="11" t="str">
-        <x:v>recipes-phosphor/configuration/entity-manager/ceb-gnrd.json</x:v>
+        <x:v>recipes-phosphor/configuration/entity-manager/ceb-gnrd.json；recipes-phosphor/psu/files/ceb-gnrd-psu-detect.sh</x:v>
       </x:c>
       <x:c r="I139"/>
       <x:c r="J139"/>
     </x:row>
-    <x:row r="140" ht="42" customHeight="1">
+    <x:row r="140" ht="52" customHeight="1">
       <x:c r="A140" s="11" t="str">
         <x:v>I2C 器件</x:v>
       </x:c>
@@ -4238,18 +4254,18 @@
         <x:v>0x59</x:v>
       </x:c>
       <x:c r="F140" s="11" t="str">
-        <x:v>PMBus；vin / vout1 / pin / pout1 / temp2</x:v>
+        <x:v>PMBus 100 kbit/s；MEG 型号专用驱动，其余 generic pmbus；仅在位地址实例化</x:v>
       </x:c>
       <x:c r="G140" s="11" t="str">
-        <x:v>PSU 电压、电功率与温度采样</x:v>
+        <x:v>PSU 电压、电功率与温度采样；实际通道由模块决定</x:v>
       </x:c>
       <x:c r="H140" s="11" t="str">
-        <x:v>recipes-phosphor/configuration/entity-manager/ceb-gnrd.json</x:v>
+        <x:v>recipes-phosphor/configuration/entity-manager/ceb-gnrd.json；recipes-phosphor/psu/files/ceb-gnrd-psu-detect.sh</x:v>
       </x:c>
       <x:c r="I140"/>
       <x:c r="J140"/>
     </x:row>
-    <x:row r="141" ht="42" customHeight="1">
+    <x:row r="141" ht="52" customHeight="1">
       <x:c r="A141" s="11" t="str">
         <x:v>I2C 器件</x:v>
       </x:c>
@@ -4266,13 +4282,13 @@
         <x:v>0x5a</x:v>
       </x:c>
       <x:c r="F141" s="11" t="str">
-        <x:v>PMBus；vin / vout1 / pin / pout1 / temp2</x:v>
+        <x:v>PMBus 100 kbit/s；MEG 型号专用驱动，其余 generic pmbus；仅在位地址实例化</x:v>
       </x:c>
       <x:c r="G141" s="11" t="str">
-        <x:v>PSU 电压、电功率与温度采样</x:v>
+        <x:v>PSU 电压、电功率与温度采样；实际通道由模块决定</x:v>
       </x:c>
       <x:c r="H141" s="11" t="str">
-        <x:v>recipes-phosphor/configuration/entity-manager/ceb-gnrd.json</x:v>
+        <x:v>recipes-phosphor/configuration/entity-manager/ceb-gnrd.json；recipes-phosphor/psu/files/ceb-gnrd-psu-detect.sh</x:v>
       </x:c>
       <x:c r="I141"/>
       <x:c r="J141"/>
@@ -4409,7 +4425,7 @@
         <x:v>VUART1 启用；IRQ 高有效；115200 baud；Linux ttyS5 / ttyVUART0</x:v>
       </x:c>
       <x:c r="G146" s="11" t="str">
-        <x:v>主机 COM1 over eSPI，用于 SOL</x:v>
+        <x:v>可选主机 COM1 over eSPI SOL；默认 SOL 为物理 UART3</x:v>
       </x:c>
       <x:c r="H146" s="11" t="str">
         <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；recipes-phosphor/console/files/server.ttyVUART0.conf</x:v>
@@ -4443,7 +4459,7 @@
       <x:c r="I147"/>
       <x:c r="J147"/>
     </x:row>
-    <x:row r="148" ht="66" customHeight="1">
+    <x:row r="148" ht="80" customHeight="1">
       <x:c r="A148" s="19" t="str">
         <x:v>DDR / 内存</x:v>
       </x:c>
@@ -4466,12 +4482,12 @@
         <x:v>BMC 系统内存</x:v>
       </x:c>
       <x:c r="H148" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；recipes-bsp/u-boot/files/ceb-gnrd-ddr4.cfg</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；recipes-bsp/u-boot/files/ceb-gnrd-ddr4.cfg</x:v>
       </x:c>
       <x:c r="I148"/>
       <x:c r="J148"/>
     </x:row>
-    <x:row r="149" ht="52" customHeight="1">
+    <x:row r="149" ht="66" customHeight="1">
       <x:c r="A149" s="11" t="str">
         <x:v>DDR / 内存</x:v>
       </x:c>
@@ -4492,7 +4508,7 @@
         <x:v>配置 DDR 工作速率</x:v>
       </x:c>
       <x:c r="H149" s="11" t="str">
-        <x:v>U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts；recipes-bsp/u-boot/files/ceb-gnrd-ddr4.cfg</x:v>
+        <x:v>U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；recipes-bsp/u-boot/files/ceb-gnrd-ddr4.cfg</x:v>
       </x:c>
       <x:c r="I149"/>
       <x:c r="J149"/>
@@ -4523,7 +4539,7 @@
       <x:c r="I150"/>
       <x:c r="J150"/>
     </x:row>
-    <x:row r="151" ht="52" customHeight="1">
+    <x:row r="151" ht="66" customHeight="1">
       <x:c r="A151" s="11" t="str">
         <x:v>DDR / 内存</x:v>
       </x:c>
@@ -4544,7 +4560,7 @@
         <x:v>内存初始化及容量配置</x:v>
       </x:c>
       <x:c r="H151" s="11" t="str">
-        <x:v>recipes-bsp/u-boot/files/ceb-gnrd-ddr4.cfg；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>recipes-bsp/u-boot/files/ceb-gnrd-ddr4.cfg；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I151"/>
       <x:c r="J151"/>
@@ -4601,7 +4617,7 @@
       <x:c r="I153"/>
       <x:c r="J153"/>
     </x:row>
-    <x:row r="154" ht="52" customHeight="1">
+    <x:row r="154" ht="66" customHeight="1">
       <x:c r="A154" s="19" t="str">
         <x:v>Flash 分区</x:v>
       </x:c>
@@ -4624,12 +4640,12 @@
         <x:v>启动引导程序</x:v>
       </x:c>
       <x:c r="H154" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I154"/>
       <x:c r="J154"/>
     </x:row>
-    <x:row r="155" ht="52" customHeight="1">
+    <x:row r="155" ht="66" customHeight="1">
       <x:c r="A155" s="11" t="str">
         <x:v>Flash 分区</x:v>
       </x:c>
@@ -4652,12 +4668,12 @@
         <x:v>U-Boot 环境存储</x:v>
       </x:c>
       <x:c r="H155" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I155"/>
       <x:c r="J155"/>
     </x:row>
-    <x:row r="156" ht="52" customHeight="1">
+    <x:row r="156" ht="66" customHeight="1">
       <x:c r="A156" s="11" t="str">
         <x:v>Flash 分区</x:v>
       </x:c>
@@ -4680,12 +4696,12 @@
         <x:v>Linux 内核</x:v>
       </x:c>
       <x:c r="H156" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I156"/>
       <x:c r="J156"/>
     </x:row>
-    <x:row r="157" ht="52" customHeight="1">
+    <x:row r="157" ht="80" customHeight="1">
       <x:c r="A157" s="11" t="str">
         <x:v>Flash 分区</x:v>
       </x:c>
@@ -4702,18 +4718,18 @@
         <x:v>offset=0x00a00000</x:v>
       </x:c>
       <x:c r="F157" s="11" t="str">
-        <x:v>size=0x02c00000（44 MiB）</x:v>
+        <x:v>size=0x02800000（40 MiB）；SquashFS-XZ</x:v>
       </x:c>
       <x:c r="G157" s="11" t="str">
         <x:v>只读文件系统</x:v>
       </x:c>
       <x:c r="H157" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；conf/machine/ceb-gnrd.conf</x:v>
       </x:c>
       <x:c r="I157"/>
       <x:c r="J157"/>
     </x:row>
-    <x:row r="158" ht="52" customHeight="1">
+    <x:row r="158" ht="80" customHeight="1">
       <x:c r="A158" s="11" t="str">
         <x:v>Flash 分区</x:v>
       </x:c>
@@ -4727,16 +4743,16 @@
         <x:v>BMC 64 MiB SPI NOR</x:v>
       </x:c>
       <x:c r="E158" s="11" t="str">
-        <x:v>offset=0x03600000</x:v>
+        <x:v>offset=0x03200000</x:v>
       </x:c>
       <x:c r="F158" s="11" t="str">
-        <x:v>size=0x00a00000（10 MiB）</x:v>
+        <x:v>size=0x00e00000（14 MiB）；JFFS2</x:v>
       </x:c>
       <x:c r="G158" s="11" t="str">
         <x:v>可写持久存储</x:v>
       </x:c>
       <x:c r="H158" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch；conf/machine/ceb-gnrd.conf</x:v>
       </x:c>
       <x:c r="I158"/>
       <x:c r="J158"/>
@@ -4769,7 +4785,7 @@
       <x:c r="I159"/>
       <x:c r="J159"/>
     </x:row>
-    <x:row r="160" ht="52" customHeight="1">
+    <x:row r="160" ht="66" customHeight="1">
       <x:c r="A160" s="19" t="str">
         <x:v>禁用 / 预留</x:v>
       </x:c>
@@ -4790,7 +4806,7 @@
         <x:v>未使用的网口资源</x:v>
       </x:c>
       <x:c r="H160" s="18" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I160"/>
       <x:c r="J160"/>
@@ -4821,7 +4837,7 @@
       <x:c r="I161"/>
       <x:c r="J161"/>
     </x:row>
-    <x:row r="162" ht="52" customHeight="1">
+    <x:row r="162" ht="66" customHeight="1">
       <x:c r="A162" s="11" t="str">
         <x:v>禁用 / 预留</x:v>
       </x:c>
@@ -4842,12 +4858,12 @@
         <x:v>未使用的存储接口</x:v>
       </x:c>
       <x:c r="H162" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I162"/>
       <x:c r="J162"/>
     </x:row>
-    <x:row r="163" ht="52" customHeight="1">
+    <x:row r="163" ht="66" customHeight="1">
       <x:c r="A163" s="11" t="str">
         <x:v>禁用 / 预留</x:v>
       </x:c>
@@ -4868,10 +4884,36 @@
         <x:v>保留 GPIOM1 给 Flash 选择信号</x:v>
       </x:c>
       <x:c r="H163" s="11" t="str">
-        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot: recipes-bsp/u-boot/files/ast2600-ceb-gnrd.dts</x:v>
+        <x:v>Linux: recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；U-Boot DTS: recipes-bsp/u-boot/files/0001-ceb-gnrd-board-device-tree-network-and-environment.patch</x:v>
       </x:c>
       <x:c r="I163"/>
       <x:c r="J163"/>
+    </x:row>
+    <x:row r="164" ht="125" customHeight="1">
+      <x:c r="A164" s="24" t="str">
+        <x:v>JTAG / CPLD</x:v>
+      </x:c>
+      <x:c r="B164" s="24" t="str">
+        <x:v>JTAG Master-1</x:v>
+      </x:c>
+      <x:c r="C164" s="23" t="str">
+        <x:v>AST2600 专用 Master-1；球位 B9/A9/D9/C9</x:v>
+      </x:c>
+      <x:c r="D164" s="23" t="str">
+        <x:v>板级 CPLD</x:v>
+      </x:c>
+      <x:c r="E164" s="23" t="str">
+        <x:v>寄存器 0x1e6e4000 / 0x40</x:v>
+      </x:c>
+      <x:c r="F164" s="23" t="str">
+        <x:v>专用 Master-1 clocks/reset；不选择 GPIOI Master-2 pinctrl</x:v>
+      </x:c>
+      <x:c r="G164" s="23" t="str">
+        <x:v>CPLD 在线编程及 Flash 读回</x:v>
+      </x:c>
+      <x:c r="H164" s="23" t="str">
+        <x:v>recipes-kernel/linux/files/aspeed-ceb-gnrd.dts；recipes-kernel/linux/files/ceb-gnrd-jtag.c</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4880,7 +4922,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R003f58225c8d443c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9232d65d77194a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>